<commit_message>
[IMP] new testenv version
</commit_message>
<xml_diff>
--- a/test_testenv/tests/data/account_tax.xlsx
+++ b/test_testenv/tests/data/account_tax.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="109">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -64,6 +64,15 @@
     <t xml:space="preserve">rc</t>
   </si>
   <si>
+    <t xml:space="preserve">rc_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rc_sale_tax_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">payability</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.tax_22a</t>
   </si>
   <si>
@@ -127,6 +136,12 @@
     <t xml:space="preserve">l10n_it_ade.n6_6</t>
   </si>
   <si>
+    <t xml:space="preserve">self</t>
+  </si>
+  <si>
+    <t xml:space="preserve">z0bug.tax_aa17c6cv</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.tax_a17c6cv</t>
   </si>
   <si>
@@ -142,9 +157,6 @@
     <t xml:space="preserve">Art.17 c.6 lett. C DPR633 (Elettronici)</t>
   </si>
   <si>
-    <t xml:space="preserve">z0bug.tax_aa17c6cv</t>
-  </si>
-  <si>
     <t xml:space="preserve">aa17c6cv</t>
   </si>
   <si>
@@ -217,6 +229,9 @@
     <t xml:space="preserve">Acq.N.I. art.8a DPR633 (Dogana)</t>
   </si>
   <si>
+    <t xml:space="preserve">z0bug.tax_aa8av</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.tax_a8av</t>
   </si>
   <si>
@@ -226,9 +241,6 @@
     <t xml:space="preserve">Vend.N.I. art.8a DPR633 (Dogana)</t>
   </si>
   <si>
-    <t xml:space="preserve">z0bug.tax_aa8av</t>
-  </si>
-  <si>
     <t xml:space="preserve">aa8av</t>
   </si>
   <si>
@@ -322,6 +334,9 @@
     <t xml:space="preserve">Acq. (RC 22%) N.I. art.17 c.2 DPR633</t>
   </si>
   <si>
+    <t xml:space="preserve">z0bug.tax_aa17c2v</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.tax_a17c2v</t>
   </si>
   <si>
@@ -329,9 +344,6 @@
   </si>
   <si>
     <t xml:space="preserve">Vend. (RC 22%) N.I. art.17 c.2 DPR633</t>
-  </si>
-  <si>
-    <t xml:space="preserve">z0bug.tax_aa17c2v</t>
   </si>
   <si>
     <t xml:space="preserve">aa17c2v</t>
@@ -348,7 +360,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -375,6 +387,11 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -419,7 +436,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -438,6 +455,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -576,7 +597,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.29"/>
@@ -590,6 +611,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="23.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="25.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="32.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13.07"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -632,16 +655,25 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>1</v>
@@ -650,30 +682,30 @@
         <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>1</v>
@@ -682,30 +714,30 @@
         <v>22</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>10</v>
@@ -714,30 +746,30 @@
         <v>22</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>20</v>
@@ -746,36 +778,42 @@
         <v>22</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>20</v>
@@ -784,36 +822,39 @@
         <v>22</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>21</v>
@@ -822,34 +863,34 @@
         <v>22</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="M7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>30</v>
@@ -858,36 +899,39 @@
         <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>30</v>
@@ -896,33 +940,39 @@
         <v>0</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>31</v>
@@ -931,33 +981,33 @@
         <v>22</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>35</v>
@@ -966,24 +1016,25 @@
         <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="N11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>35</v>
@@ -992,30 +1043,30 @@
         <v>0</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>40</v>
@@ -1024,36 +1075,42 @@
         <v>22</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D14" s="1" t="n">
         <v>40</v>
@@ -1062,26 +1119,26 @@
         <v>0</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>41</v>
@@ -1090,30 +1147,30 @@
         <v>22</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D16" s="1" t="n">
         <v>50</v>
@@ -1122,24 +1179,24 @@
         <v>0</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D17" s="1" t="n">
         <v>50</v>
@@ -1148,24 +1205,24 @@
         <v>0</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>60</v>
@@ -1174,24 +1231,24 @@
         <v>0</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>60</v>
@@ -1200,24 +1257,24 @@
         <v>0</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D20" s="1" t="n">
         <v>60</v>
@@ -1226,24 +1283,24 @@
         <v>0</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D21" s="1" t="n">
         <v>60</v>
@@ -1252,24 +1309,24 @@
         <v>0</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>60</v>
@@ -1278,27 +1335,27 @@
         <v>0</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D23" s="1" t="n">
         <v>60</v>
@@ -1307,30 +1364,30 @@
         <v>0</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>80</v>
@@ -1339,36 +1396,42 @@
         <v>22</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D25" s="1" t="n">
         <v>80</v>
@@ -1377,33 +1440,33 @@
         <v>22</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>81</v>
@@ -1412,19 +1475,19 @@
         <v>22</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>